<commit_message>
fix: 修复 info_database.xlsx 数据格式并添加表头冻结 Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/info_database.xlsx
+++ b/resources/userdata/info_database.xlsx
@@ -3089,7 +3089,6 @@
           <t>拉丁裔,</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr"/>
       <c r="D122" t="inlineStr">
         <is>
           <t>,拉丁裔,拉丁美女,ラティーナ,</t>
@@ -8350,7 +8349,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>精液狂热,スペルママニア,マンコぶっかけ,外射,射在外阴,射在外陰,阴部射精,射在衣服上,着衣に精液,衣物沾精液,射在胸部,胸に精液,胸口精液,大腿上的精液,太腿に精液,射在大腿,射在屁股,尻に精液,精液沾臀,精液塗り込み,精液塗抹,精液涂抹,精液交换,精液交換,射在腹部,腹に精液,腹部精液,头发沾精液,射在頭髮,髪に精液,</t>
+          <t>,精液狂热,スペルママニア,マンコぶっかけ,外射,射在外阴,射在外陰,阴部射精,射在衣服上,着衣に精液,衣物沾精液,射在胸部,胸に精液,胸口精液,大腿上的精液,太腿に精液,射在大腿,射在屁股,尻に精液,精液沾臀,精液塗り込み,精液塗抹,精液涂抹,精液交换,精液交換,射在腹部,腹に精液,腹部精液,头发沾精液,射在頭髮,髪に精液,</t>
         </is>
       </c>
     </row>
@@ -8680,7 +8679,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>礼仪小姐,禮儀小姐,</t>
+          <t>,礼仪小姐,禮儀小姐,</t>
         </is>
       </c>
     </row>
@@ -11166,7 +11165,7 @@
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>ハヤブサ,</t>
+          <t>,ハヤブサ,</t>
         </is>
       </c>
     </row>
@@ -12293,9 +12292,11 @@
       </c>
     </row>
     <row r="541">
-      <c r="A541" t="inlineStr"/>
-      <c r="B541" t="inlineStr"/>
-      <c r="C541" t="inlineStr"/>
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>えむっ娘ラボ</t>
+        </is>
+      </c>
       <c r="D541" t="inlineStr">
         <is>
           <t>,えむっ娘ラボ,</t>
@@ -15928,7 +15929,7 @@
       </c>
       <c r="D706" t="inlineStr">
         <is>
-          <t>素人しか勝たん,</t>
+          <t>,素人しか勝たん,</t>
         </is>
       </c>
     </row>

</xml_diff>